<commit_message>
refactor: adapt parse_row to web structure changes
- Fix: Adapt parse_row() to handle dynamic HTML row lengths
  * Address structural updates where row elements fluctuated from 28 to 28-30.
  * Implement keyword-based exclusion (EXCLUDED_KEYWORDS) to strip randomly inserted metadata (e.g., "健康", "電影").
  * Stabilize indexing by normalizing the parts list before iterative parsing.
- Refactor: Improve code robustness and formatting
  * Standardize global variable declarations and enhance inline documentation.
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="113-1" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="113-2" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="114-1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="114-2" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1271,4 +1272,174 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>星期一 Mon</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>星期二 Tue</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>星期三 Wed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>星期四 Thr</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>星期五 Fri</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1830-1915</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>空堂 - Free Period</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>資訊安全 - Information Security</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>人工智慧 - Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>電腦視覺應用 - Computer Vision and Application</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>數位行銷與品牌 - Digital Marketing and Branding</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1915-2000</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>空堂 - Free Period</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>資訊安全 - Information Security</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>人工智慧 - Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>電腦視覺應用 - Computer Vision and Application</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>數位行銷與品牌 - Digital Marketing and Branding</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2010-2055</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>空堂 - Free Period</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>資訊安全 - Information Security</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>人工智慧 - Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>電腦視覺應用 - Computer Vision and Application</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>數位行銷與品牌 - Digital Marketing and Branding</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2055-2140</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>空堂 - Free Period</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>空堂 - Free Period</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>空堂 - Free Period</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>空堂 - Free Period</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>空堂 - Free Period</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>